<commit_message>
EG-49 Improved CC1101 registers settings from new baudrate calculation.
</commit_message>
<xml_diff>
--- a/docs/references/datasheets/sensor/CC1101.xlsx
+++ b/docs/references/datasheets/sensor/CC1101.xlsx
@@ -8,7 +8,8 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="433" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="868" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="13">
   <si>
     <t xml:space="preserve">MHz</t>
   </si>
@@ -69,11 +70,12 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -89,6 +91,11 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -133,21 +140,29 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -276,124 +291,128 @@
   <dimension ref="A2:D22"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.07"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="2" t="n">
         <v>433.92</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="3" t="str">
+      <c r="B5" s="4" t="str">
         <f aca="false">DEC2HEX(MOD(INT((B2*1000000)/((B3*1000000)/2^16) / 65536), 256))</f>
         <v>10</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="3" t="str">
+      <c r="B6" s="4" t="str">
         <f aca="false">DEC2HEX(MOD(INT((B2*1000000)/((B3*1000000)/2^16)/ 256), 256))</f>
         <v>B0</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="3" t="str">
+      <c r="B7" s="4" t="str">
         <f aca="false">DEC2HEX(MOD((B2*1000000)/((B3*1000000)/2^16),256))</f>
         <v>71</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="3" t="str">
+      <c r="B9" s="4" t="str">
         <f aca="false">DEC2HEX((B2*1000000)/((B3*1000000)/2^16))</f>
         <v>10B071</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="1" t="n">
         <f aca="false">(B3*1000000)/(8*(4+B16)*2^B15)/1000</f>
-        <v>203.125</v>
-      </c>
-      <c r="C13" s="0" t="s">
+        <v>101.5625</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C15" s="0" t="s">
+      <c r="A15" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" s="0" t="n">
+      <c r="A16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="1" t="n">
         <f aca="false">((((256+B22)*2^B21)*B3*1000000)/2^28)/1000</f>
         <v>1.25217437744141</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="C21" s="0" t="s">
+      <c r="B21" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="D21" s="5" t="str">
+        <f aca="false">DEC2HEX(B21)</f>
+        <v>5</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="1" t="n">
         <v>148</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="0" t="str">
+      <c r="D22" s="1" t="str">
         <f aca="false">DEC2HEX(B22)</f>
         <v>94</v>
       </c>
@@ -407,4 +426,149 @@
     <oddFooter>&amp;CPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A2:D22"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.07"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="n">
+        <v>868.5</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B3" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="4" t="str">
+        <f aca="false">DEC2HEX(MOD(INT((B2*1000000)/((B3*1000000)/2^16) / 65536), 256))</f>
+        <v>21</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="4" t="str">
+        <f aca="false">DEC2HEX(MOD(INT((B2*1000000)/((B3*1000000)/2^16)/ 256), 256))</f>
+        <v>67</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="4" t="str">
+        <f aca="false">DEC2HEX(MOD((B2*1000000)/((B3*1000000)/2^16),256))</f>
+        <v>62</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="4" t="str">
+        <f aca="false">DEC2HEX((B2*1000000)/((B3*1000000)/2^16))</f>
+        <v>216762</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="1" t="n">
+        <f aca="false">(B3*1000000)/(8*(4+B16)*2^B15)/1000</f>
+        <v>101.5625</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="1" t="n">
+        <f aca="false">((((256+B22)*2^B21)*B3*1000000)/2^28)/1000</f>
+        <v>1.25217437744141</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="5" t="str">
+        <f aca="false">DEC2HEX(B21)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>148</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="1" t="str">
+        <f aca="false">DEC2HEX(B22)</f>
+        <v>94</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;A</oddHeader>
+    <oddFooter>&amp;CPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>